<commit_message>
Format code and improve product title extraction
Refactor index.ts with consistent formatting and line breaks for improved readability. Use page H1 as output title instead of search result title for more accurate product representation. Update Reebelo service to properly return and handle selectedCondition in matchDirectly method.
</commit_message>
<xml_diff>
--- a/output/amazon_2026-06-30.xlsx
+++ b/output/amazon_2026-06-30.xlsx
@@ -477,16 +477,16 @@
         <v>Apple iPhone 12 Pro 5G (128GB, Blue) - Excellent</v>
       </c>
       <c r="C3" t="str">
-        <v>https://www.amazon.com.au/dp/B098P7QYFL</v>
+        <v>https://www.amazon.com.au/dp/B0968GVWLZ</v>
       </c>
       <c r="D3" t="str">
-        <v>128GB, 128 GB, 128GB, 128 GB | Pacific Blue</v>
+        <v>128GB, 128 GB, 128GB, 128 GB | Gold</v>
       </c>
       <c r="E3" t="str">
-        <v>395</v>
+        <v>414</v>
       </c>
       <c r="F3" t="str">
-        <v>iPhone 12 Pro 128GB Pacific Blue (Renewed)</v>
+        <v>Filter by</v>
       </c>
       <c r="G3" t="str">
         <v>0.5</v>
@@ -501,7 +501,7 @@
         <v>Excellent</v>
       </c>
       <c r="K3" t="str">
-        <v>https://www.amazon.com.au/dp/B098P7QYFL</v>
+        <v>https://www.amazon.com.au/dp/B0968GVWLZ</v>
       </c>
     </row>
     <row r="4">
@@ -609,7 +609,7 @@
         <v/>
       </c>
     </row>
-    <row r="7">
+    <row r="7" xml:space="preserve">
       <c r="A7" t="str">
         <v>iPhone12Pro5G128GBSilv-RD-VR-EXD-AU</v>
       </c>
@@ -617,34 +617,41 @@
         <v>Apple iPhone 12 Pro 5G (128GB, Silver) - Excellent</v>
       </c>
       <c r="C7" t="str">
-        <v/>
+        <v>https://www.amazon.com.au/dp/B0968GVWLZ</v>
       </c>
       <c r="D7" t="str">
-        <v/>
+        <v>128GB, 128 GB, 128GB, 128 GB | Gold</v>
       </c>
       <c r="E7" t="str">
-        <v/>
-      </c>
-      <c r="F7" t="str">
-        <v/>
+        <v>414</v>
+      </c>
+      <c r="F7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Product summary presents key product information       Keyboard shortcut  
+                        Shift
+                        +
+                         Alt
+                        +
+                        opt
+                        +
+                        D</v>
       </c>
       <c r="G7" t="str">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H7" t="str">
-        <v>no_match</v>
+        <v>matched</v>
       </c>
       <c r="I7" t="str">
         <v/>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>Excellent</v>
       </c>
       <c r="K7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
+        <v>https://www.amazon.com.au/dp/B0968GVWLZ</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
       <c r="A8" t="str">
         <v>iP12Pro5G256GBBlue-RD-VR-EXD-AU</v>
       </c>
@@ -652,31 +659,38 @@
         <v>Apple iPhone 12 Pro 5G (256GB, Blue) - Excellent</v>
       </c>
       <c r="C8" t="str">
-        <v/>
+        <v>https://www.amazon.com.au/dp/B0968GVWLZ</v>
       </c>
       <c r="D8" t="str">
-        <v/>
+        <v>128GB, 128 GB, 128GB, 128 GB | Gold</v>
       </c>
       <c r="E8" t="str">
-        <v/>
-      </c>
-      <c r="F8" t="str">
-        <v/>
+        <v>414</v>
+      </c>
+      <c r="F8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Product summary presents key product information       Keyboard shortcut  
+                        Shift
+                        +
+                         Alt
+                        +
+                        opt
+                        +
+                        D</v>
       </c>
       <c r="G8" t="str">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H8" t="str">
-        <v>no_match</v>
+        <v>matched</v>
       </c>
       <c r="I8" t="str">
         <v/>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>Excellent</v>
       </c>
       <c r="K8" t="str">
-        <v/>
+        <v>https://www.amazon.com.au/dp/B0968GVWLZ</v>
       </c>
     </row>
     <row r="9">

</xml_diff>